<commit_message>
fix: address Grok character rule findings
</commit_message>
<xml_diff>
--- a/docs/verification/style-guide-licensing-review-20260727/character-franchise-rule-audit.xlsx
+++ b/docs/verification/style-guide-licensing-review-20260727/character-franchise-rule-audit.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule audit" sheetId="1" r:id="Rd74f160a7db04204"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R6fa07fe4f3834091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule audit" sheetId="1" r:id="R857f4f8e41bd49e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rddd0d0de870a4bb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1187,13 +1187,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E26" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F26" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>GN</x:v>
       </x:c>
       <x:c r="G26" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Green Lantern character family</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
@@ -1464,7 +1464,9 @@
         <x:v>SENTINEL_EXCLUDED</x:v>
       </x:c>
       <x:c r="F38" s="69" t="str"/>
-      <x:c r="G38" s="56" t="str"/>
+      <x:c r="G38" s="56" t="str">
+        <x:v>Royalty reporting sentinel; not a canonical character</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="56" t="str">
@@ -1752,13 +1754,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E51" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F51" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>SM</x:v>
       </x:c>
       <x:c r="G51" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Superman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
@@ -1775,13 +1777,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E52" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F52" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>FS</x:v>
       </x:c>
       <x:c r="G52" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Flash character family</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
@@ -1867,13 +1869,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E56" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F56" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>WW</x:v>
       </x:c>
       <x:c r="G56" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Wonder Woman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
@@ -2029,7 +2031,9 @@
         <x:v>SENTINEL_EXCLUDED</x:v>
       </x:c>
       <x:c r="F63" s="69" t="str"/>
-      <x:c r="G63" s="56" t="str"/>
+      <x:c r="G63" s="56" t="str">
+        <x:v>Royalty reporting sentinel; not a canonical character</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="56" t="str">
@@ -2137,13 +2141,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E68" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F68" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>WW</x:v>
       </x:c>
       <x:c r="G68" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Wonder Woman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
@@ -2158,13 +2162,11 @@
       </x:c>
       <x:c r="D69" s="56" t="str"/>
       <x:c r="E69" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F69" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F69" s="69" t="str"/>
       <x:c r="G69" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
@@ -2410,13 +2412,11 @@
       </x:c>
       <x:c r="D81" s="56" t="str"/>
       <x:c r="E81" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F81" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F81" s="69" t="str"/>
       <x:c r="G81" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
@@ -2641,13 +2641,13 @@
       </x:c>
       <x:c r="D92" s="56" t="str"/>
       <x:c r="E92" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F92" s="69" t="str">
-        <x:v>SP</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G92" s="56" t="str">
-        <x:v>Spider-Man character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
@@ -3733,13 +3733,11 @@
       </x:c>
       <x:c r="D144" s="56" t="str"/>
       <x:c r="E144" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F144" s="69" t="str">
-        <x:v>GG</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F144" s="69" t="str"/>
       <x:c r="G144" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
@@ -4867,13 +4865,11 @@
       </x:c>
       <x:c r="D198" s="56" t="str"/>
       <x:c r="E198" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F198" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F198" s="69" t="str"/>
       <x:c r="G198" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
@@ -4909,13 +4905,11 @@
       </x:c>
       <x:c r="D200" s="56" t="str"/>
       <x:c r="E200" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F200" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F200" s="69" t="str"/>
       <x:c r="G200" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
@@ -4930,13 +4924,11 @@
       </x:c>
       <x:c r="D201" s="56" t="str"/>
       <x:c r="E201" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F201" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F201" s="69" t="str"/>
       <x:c r="G201" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="22" customHeight="1">
@@ -4951,13 +4943,11 @@
       </x:c>
       <x:c r="D202" s="56" t="str"/>
       <x:c r="E202" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F202" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F202" s="69" t="str"/>
       <x:c r="G202" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="22" customHeight="1">
@@ -4972,13 +4962,11 @@
       </x:c>
       <x:c r="D203" s="56" t="str"/>
       <x:c r="E203" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F203" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F203" s="69" t="str"/>
       <x:c r="G203" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="22" customHeight="1">
@@ -4993,13 +4981,13 @@
       </x:c>
       <x:c r="D204" s="56" t="str"/>
       <x:c r="E204" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F204" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G204" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="22" customHeight="1">
@@ -5014,13 +5002,13 @@
       </x:c>
       <x:c r="D205" s="56" t="str"/>
       <x:c r="E205" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F205" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G205" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="22" customHeight="1">
@@ -5623,13 +5611,13 @@
       </x:c>
       <x:c r="D234" s="56" t="str"/>
       <x:c r="E234" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F234" s="69" t="str">
-        <x:v>GG</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G234" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="22" customHeight="1">
@@ -5644,13 +5632,13 @@
       </x:c>
       <x:c r="D235" s="56" t="str"/>
       <x:c r="E235" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F235" s="69" t="str">
-        <x:v>GG</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G235" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="22" customHeight="1">
@@ -6442,13 +6430,13 @@
       </x:c>
       <x:c r="D273" s="56" t="str"/>
       <x:c r="E273" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F273" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G273" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="274" ht="22" customHeight="1">
@@ -6463,13 +6451,13 @@
       </x:c>
       <x:c r="D274" s="56" t="str"/>
       <x:c r="E274" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F274" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G274" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="275" ht="22" customHeight="1">
@@ -7555,13 +7543,13 @@
       </x:c>
       <x:c r="D326" s="56" t="str"/>
       <x:c r="E326" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F326" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G326" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="327" ht="22" customHeight="1">
@@ -7744,13 +7732,11 @@
       </x:c>
       <x:c r="D335" s="56" t="str"/>
       <x:c r="E335" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F335" s="69" t="str">
-        <x:v>XM</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F335" s="69" t="str"/>
       <x:c r="G335" s="56" t="str">
-        <x:v>X-Men character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="336" ht="22" customHeight="1">
@@ -7843,7 +7829,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf14a596e404b4f47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcec68325e58844e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7883,7 +7869,7 @@
         <x:v>Specific franchise rules</x:v>
       </x:c>
       <x:c r="B5" s="36" t="n">
-        <x:v>256</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -7891,7 +7877,7 @@
         <x:v>Existing unique matches</x:v>
       </x:c>
       <x:c r="B6" s="36" t="n">
-        <x:v>18</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -7899,14 +7885,22 @@
         <x:v>Marvel catch-all</x:v>
       </x:c>
       <x:c r="B7" s="36" t="n">
-        <x:v>62</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="28" t="str">
+      <x:c r="A8" s="26" t="str">
+        <x:v>Non-character labels excluded</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="28" t="str">
         <x:v>Licensing follow-up rows</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="n">
+      <x:c r="B9" s="37" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix: address Grok character rule findings (#267)
Co-authored-by: Albert Hazan <u2giants@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/verification/style-guide-licensing-review-20260727/character-franchise-rule-audit.xlsx
+++ b/docs/verification/style-guide-licensing-review-20260727/character-franchise-rule-audit.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule audit" sheetId="1" r:id="Rd74f160a7db04204"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="R6fa07fe4f3834091"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rule audit" sheetId="1" r:id="R857f4f8e41bd49e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" r:id="Rddd0d0de870a4bb3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1187,13 +1187,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E26" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F26" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>GN</x:v>
       </x:c>
       <x:c r="G26" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Green Lantern character family</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="22" customHeight="1">
@@ -1464,7 +1464,9 @@
         <x:v>SENTINEL_EXCLUDED</x:v>
       </x:c>
       <x:c r="F38" s="69" t="str"/>
-      <x:c r="G38" s="56" t="str"/>
+      <x:c r="G38" s="56" t="str">
+        <x:v>Royalty reporting sentinel; not a canonical character</x:v>
+      </x:c>
     </x:row>
     <x:row r="39" ht="22" customHeight="1">
       <x:c r="A39" s="56" t="str">
@@ -1752,13 +1754,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E51" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F51" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>SM</x:v>
       </x:c>
       <x:c r="G51" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Superman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="22" customHeight="1">
@@ -1775,13 +1777,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E52" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F52" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>FS</x:v>
       </x:c>
       <x:c r="G52" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Flash character family</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="22" customHeight="1">
@@ -1867,13 +1869,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E56" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F56" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>WW</x:v>
       </x:c>
       <x:c r="G56" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Wonder Woman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="22" customHeight="1">
@@ -2029,7 +2031,9 @@
         <x:v>SENTINEL_EXCLUDED</x:v>
       </x:c>
       <x:c r="F63" s="69" t="str"/>
-      <x:c r="G63" s="56" t="str"/>
+      <x:c r="G63" s="56" t="str">
+        <x:v>Royalty reporting sentinel; not a canonical character</x:v>
+      </x:c>
     </x:row>
     <x:row r="64" ht="22" customHeight="1">
       <x:c r="A64" s="56" t="str">
@@ -2137,13 +2141,13 @@
         <x:v>JG</x:v>
       </x:c>
       <x:c r="E68" s="56" t="str">
-        <x:v>AUTO_UNIQUE</x:v>
+        <x:v>SPECIFIC_FRANCHISE</x:v>
       </x:c>
       <x:c r="F68" s="69" t="str">
-        <x:v>JG</x:v>
+        <x:v>WW</x:v>
       </x:c>
       <x:c r="G68" s="56" t="str">
-        <x:v>One unique same-licensor property found in already resolved style guides</x:v>
+        <x:v>Wonder Woman character family</x:v>
       </x:c>
     </x:row>
     <x:row r="69" ht="22" customHeight="1">
@@ -2158,13 +2162,11 @@
       </x:c>
       <x:c r="D69" s="56" t="str"/>
       <x:c r="E69" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F69" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F69" s="69" t="str"/>
       <x:c r="G69" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="70" ht="22" customHeight="1">
@@ -2410,13 +2412,11 @@
       </x:c>
       <x:c r="D81" s="56" t="str"/>
       <x:c r="E81" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F81" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F81" s="69" t="str"/>
       <x:c r="G81" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="82" ht="22" customHeight="1">
@@ -2641,13 +2641,13 @@
       </x:c>
       <x:c r="D92" s="56" t="str"/>
       <x:c r="E92" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F92" s="69" t="str">
-        <x:v>SP</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G92" s="56" t="str">
-        <x:v>Spider-Man character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="93" ht="22" customHeight="1">
@@ -3733,13 +3733,11 @@
       </x:c>
       <x:c r="D144" s="56" t="str"/>
       <x:c r="E144" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F144" s="69" t="str">
-        <x:v>GG</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F144" s="69" t="str"/>
       <x:c r="G144" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="145" ht="22" customHeight="1">
@@ -4867,13 +4865,11 @@
       </x:c>
       <x:c r="D198" s="56" t="str"/>
       <x:c r="E198" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F198" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F198" s="69" t="str"/>
       <x:c r="G198" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="22" customHeight="1">
@@ -4909,13 +4905,11 @@
       </x:c>
       <x:c r="D200" s="56" t="str"/>
       <x:c r="E200" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F200" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F200" s="69" t="str"/>
       <x:c r="G200" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="201" ht="22" customHeight="1">
@@ -4930,13 +4924,11 @@
       </x:c>
       <x:c r="D201" s="56" t="str"/>
       <x:c r="E201" s="56" t="str">
-        <x:v>MARVEL_CATCH_ALL</x:v>
-      </x:c>
-      <x:c r="F201" s="69" t="str">
-        <x:v>MV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F201" s="69" t="str"/>
       <x:c r="G201" s="56" t="str">
-        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="202" ht="22" customHeight="1">
@@ -4951,13 +4943,11 @@
       </x:c>
       <x:c r="D202" s="56" t="str"/>
       <x:c r="E202" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F202" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F202" s="69" t="str"/>
       <x:c r="G202" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="203" ht="22" customHeight="1">
@@ -4972,13 +4962,11 @@
       </x:c>
       <x:c r="D203" s="56" t="str"/>
       <x:c r="E203" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F203" s="69" t="str">
-        <x:v>AV</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F203" s="69" t="str"/>
       <x:c r="G203" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="204" ht="22" customHeight="1">
@@ -4993,13 +4981,13 @@
       </x:c>
       <x:c r="D204" s="56" t="str"/>
       <x:c r="E204" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F204" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G204" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="205" ht="22" customHeight="1">
@@ -5014,13 +5002,13 @@
       </x:c>
       <x:c r="D205" s="56" t="str"/>
       <x:c r="E205" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F205" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G205" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="206" ht="22" customHeight="1">
@@ -5623,13 +5611,13 @@
       </x:c>
       <x:c r="D234" s="56" t="str"/>
       <x:c r="E234" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F234" s="69" t="str">
-        <x:v>GG</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G234" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="22" customHeight="1">
@@ -5644,13 +5632,13 @@
       </x:c>
       <x:c r="D235" s="56" t="str"/>
       <x:c r="E235" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F235" s="69" t="str">
-        <x:v>GG</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G235" s="56" t="str">
-        <x:v>Guardians of the Galaxy character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="236" ht="22" customHeight="1">
@@ -6442,13 +6430,13 @@
       </x:c>
       <x:c r="D273" s="56" t="str"/>
       <x:c r="E273" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F273" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G273" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="274" ht="22" customHeight="1">
@@ -6463,13 +6451,13 @@
       </x:c>
       <x:c r="D274" s="56" t="str"/>
       <x:c r="E274" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F274" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G274" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="275" ht="22" customHeight="1">
@@ -7555,13 +7543,13 @@
       </x:c>
       <x:c r="D326" s="56" t="str"/>
       <x:c r="E326" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
+        <x:v>MARVEL_CATCH_ALL</x:v>
       </x:c>
       <x:c r="F326" s="69" t="str">
-        <x:v>AV</x:v>
+        <x:v>MV</x:v>
       </x:c>
       <x:c r="G326" s="56" t="str">
-        <x:v>Avengers character family</x:v>
+        <x:v>Marvel Assorted Styles catch-all; no narrower current MG06 franchise rule</x:v>
       </x:c>
     </x:row>
     <x:row r="327" ht="22" customHeight="1">
@@ -7744,13 +7732,11 @@
       </x:c>
       <x:c r="D335" s="56" t="str"/>
       <x:c r="E335" s="56" t="str">
-        <x:v>SPECIFIC_FRANCHISE</x:v>
-      </x:c>
-      <x:c r="F335" s="69" t="str">
-        <x:v>XM</x:v>
-      </x:c>
+        <x:v>NON_CHARACTER_EXCLUDED</x:v>
+      </x:c>
+      <x:c r="F335" s="69" t="str"/>
       <x:c r="G335" s="56" t="str">
-        <x:v>X-Men character family</x:v>
+        <x:v>Guide, logo, or general label; not a canonical character</x:v>
       </x:c>
     </x:row>
     <x:row r="336" ht="22" customHeight="1">
@@ -7843,7 +7829,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf14a596e404b4f47"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcec68325e58844e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7883,7 +7869,7 @@
         <x:v>Specific franchise rules</x:v>
       </x:c>
       <x:c r="B5" s="36" t="n">
-        <x:v>256</x:v>
+        <x:v>248</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="28" customHeight="1">
@@ -7891,7 +7877,7 @@
         <x:v>Existing unique matches</x:v>
       </x:c>
       <x:c r="B6" s="36" t="n">
-        <x:v>18</x:v>
+        <x:v>13</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="28" customHeight="1">
@@ -7899,14 +7885,22 @@
         <x:v>Marvel catch-all</x:v>
       </x:c>
       <x:c r="B7" s="36" t="n">
-        <x:v>62</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="28" customHeight="1">
-      <x:c r="A8" s="28" t="str">
+      <x:c r="A8" s="26" t="str">
+        <x:v>Non-character labels excluded</x:v>
+      </x:c>
+      <x:c r="B8" s="36" t="n">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="28" customHeight="1">
+      <x:c r="A9" s="28" t="str">
         <x:v>Licensing follow-up rows</x:v>
       </x:c>
-      <x:c r="B8" s="37" t="n">
+      <x:c r="B9" s="37" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>